<commit_message>
feat: calibrate cabin sensor parameters and add communication latency benchmark tool
</commit_message>
<xml_diff>
--- a/backend/DanhSachMau_Mau.xlsx
+++ b/backend/DanhSachMau_Mau.xlsx
@@ -397,12 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E13"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -416,82 +417,219 @@
         <v>TestType</v>
       </c>
       <c r="D1" t="str">
-        <v>DestinationStation</v>
+        <v>Trạm đích</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Ghi chú (Nguồn)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BC10001</v>
+        <v>EM-2026-001</v>
       </c>
       <c r="B2" t="str">
         <v>Nguyễn Văn An</v>
       </c>
       <c r="C2" t="str">
-        <v>Sinh hóa máu</v>
+        <v>Máu toàn phần (Heparin) - Khí máu ABG</v>
       </c>
       <c r="D2" t="str">
-        <v>Xét Nghiệm</v>
+        <v>ST-04</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Cấp Cứu → Xét Nghiệm</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BC10002</v>
+        <v>EM-2026-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Trần Thị Bình</v>
+        <v>Trần Thị Bích</v>
       </c>
       <c r="C3" t="str">
-        <v>Vi sinh nuôi cấy</v>
+        <v>Huyết thanh - Sinh hóa (Troponin I)</v>
       </c>
       <c r="D3" t="str">
-        <v>Vi Sinh</v>
+        <v>ST-02</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Cấp Cứu → Khám Bệnh</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BC10003</v>
+        <v>EM-2026-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Lê Quốc Cường</v>
+        <v>Lê Minh Tuấn</v>
       </c>
       <c r="C4" t="str">
-        <v>PCR</v>
+        <v>Huyết tương (Citrate) - Đông máu PT/APTT</v>
       </c>
       <c r="D4" t="str">
-        <v>PCR</v>
+        <v>ST-03</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Cấp Cứu → ICU</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BC10004</v>
+        <v>OPD-2026-001</v>
       </c>
       <c r="B5" t="str">
-        <v>Phạm Mai Dung</v>
+        <v>Phạm Thị Lan</v>
       </c>
       <c r="C5" t="str">
-        <v>CBC</v>
+        <v>Máu toàn phần (EDTA) - Công thức máu CBC</v>
       </c>
       <c r="D5" t="str">
-        <v>Xét Nghiệm</v>
+        <v>ST-04</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Khám Bệnh → Xét Nghiệm</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BC10005</v>
+        <v>OPD-2026-002</v>
       </c>
       <c r="B6" t="str">
-        <v>Đoàn Minh Em</v>
+        <v>Hoàng Văn Đức</v>
       </c>
       <c r="C6" t="str">
-        <v>PCR</v>
+        <v>Huyết thanh - Sinh hóa (Glucose/HbA1c)</v>
       </c>
       <c r="D6" t="str">
+        <v>ST-01</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Khám Bệnh → Cấp Cứu</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>OPD-2026-003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Vũ Thị Hoa</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Mẫu nước tiểu - Tổng phân tích 10 thông số</v>
+      </c>
+      <c r="D7" t="str">
+        <v>ST-03</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Khám Bệnh → ICU</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ICU-2026-001</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Ngô Thị Minh</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Huyết thanh - Điện giải đồ (Na, K, Cl)</v>
+      </c>
+      <c r="D8" t="str">
         <v>ST-04</v>
+      </c>
+      <c r="E8" t="str">
+        <v>ICU → Xét Nghiệm</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ICU-2026-002</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bùi Văn Hùng</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Mẫu cấy - Cấy máu tìm vi khuẩn</v>
+      </c>
+      <c r="D9" t="str">
+        <v>ST-01</v>
+      </c>
+      <c r="E9" t="str">
+        <v>ICU → Cấp Cứu</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ICU-2026-003</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Lý Thị Thu</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Mẫu dịch - Sinh hóa dịch não tủy CSF</v>
+      </c>
+      <c r="D10" t="str">
+        <v>ST-02</v>
+      </c>
+      <c r="E10" t="str">
+        <v>ICU → Khám Bệnh</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>LAB-2026-001</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Đinh Quang Khải</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Mẫu mô - Sinh thiết tức thì (Frozen)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>ST-01</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Xét Nghiệm → Cấp Cứu</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>LAB-2026-002</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Mai Thị Xuân</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Huyết thanh - Mỡ máu (Lipid Profile)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>ST-02</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Xét Nghiệm → Khám Bệnh</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>LAB-2026-003</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Võ Minh Khoa</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Huyết thanh - Miễn dịch (Procalcitonin)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>ST-03</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Xét Nghiệm → ICU</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>